<commit_message>
Replace bundled sample estate with fictional demo data
</commit_message>
<xml_diff>
--- a/data/sample_estate_demand.xlsx
+++ b/data/sample_estate_demand.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +27,23 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,9 +58,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,191 +431,163 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X26"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="G1" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>Oct-26</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>Dec-26</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>Jan-27</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>Apr-27</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>Jul-27</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>October</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>November</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>November</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>November</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>November</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>November</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>December</t>
+          <t>Aug-27</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>LOB</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Site</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="G2" s="1" t="n">
-        <v>46244</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <v>46251</v>
-      </c>
-      <c r="I2" s="1" t="n">
-        <v>46258</v>
-      </c>
-      <c r="J2" s="1" t="n">
-        <v>46265</v>
-      </c>
-      <c r="K2" s="1" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L2" s="1" t="n">
-        <v>46279</v>
-      </c>
-      <c r="M2" s="1" t="n">
-        <v>46286</v>
-      </c>
-      <c r="N2" s="1" t="n">
-        <v>46293</v>
-      </c>
-      <c r="O2" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="P2" s="1" t="n">
-        <v>46307</v>
-      </c>
-      <c r="Q2" s="1" t="n">
-        <v>46314</v>
-      </c>
-      <c r="R2" s="1" t="n">
-        <v>46321</v>
-      </c>
-      <c r="S2" s="1" t="n">
-        <v>46328</v>
-      </c>
-      <c r="T2" s="1" t="n">
-        <v>46335</v>
-      </c>
-      <c r="U2" s="1" t="n">
-        <v>46342</v>
-      </c>
-      <c r="V2" s="1" t="n">
-        <v>46349</v>
-      </c>
-      <c r="W2" s="1" t="n">
-        <v>46356</v>
-      </c>
-      <c r="X2" s="1" t="n">
-        <v>46363</v>
+      <c r="G2" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>46327</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>46357</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>46388</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>46419</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>46539</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>46569</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>46600</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Helio</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -610,17 +597,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -629,64 +616,46 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>900</v>
+        <v>147</v>
       </c>
       <c r="H3" t="n">
-        <v>911</v>
+        <v>148</v>
       </c>
       <c r="I3" t="n">
-        <v>922</v>
+        <v>149</v>
       </c>
       <c r="J3" t="n">
-        <v>932</v>
+        <v>151</v>
       </c>
       <c r="K3" t="n">
-        <v>943</v>
+        <v>152</v>
       </c>
       <c r="L3" t="n">
-        <v>954</v>
+        <v>153</v>
       </c>
       <c r="M3" t="n">
-        <v>965</v>
+        <v>154</v>
       </c>
       <c r="N3" t="n">
-        <v>976</v>
+        <v>156</v>
       </c>
       <c r="O3" t="n">
-        <v>986</v>
+        <v>157</v>
       </c>
       <c r="P3" t="n">
-        <v>997</v>
+        <v>158</v>
       </c>
       <c r="Q3" t="n">
-        <v>1008</v>
+        <v>159</v>
       </c>
       <c r="R3" t="n">
-        <v>1019</v>
-      </c>
-      <c r="S3" t="n">
-        <v>1030</v>
-      </c>
-      <c r="T3" t="n">
-        <v>1040</v>
-      </c>
-      <c r="U3" t="n">
-        <v>1051</v>
-      </c>
-      <c r="V3" t="n">
-        <v>1062</v>
-      </c>
-      <c r="W3" t="n">
-        <v>1073</v>
-      </c>
-      <c r="X3" t="n">
-        <v>1084</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Helio</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -696,17 +665,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -715,64 +684,46 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="H4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="I4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="J4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="K4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="L4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="M4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="N4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="O4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="P4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="R4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="S4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="T4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="U4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="V4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="W4" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="X4" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Helio</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -782,17 +733,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -801,84 +752,66 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>750</v>
+        <v>127.8</v>
       </c>
       <c r="H5" t="n">
-        <v>759.17</v>
+        <v>128.7</v>
       </c>
       <c r="I5" t="n">
-        <v>768.33</v>
+        <v>129.6</v>
       </c>
       <c r="J5" t="n">
-        <v>776.67</v>
+        <v>131.3</v>
       </c>
       <c r="K5" t="n">
-        <v>785.83</v>
+        <v>132.2</v>
       </c>
       <c r="L5" t="n">
-        <v>795</v>
+        <v>133</v>
       </c>
       <c r="M5" t="n">
-        <v>804.17</v>
+        <v>133.9</v>
       </c>
       <c r="N5" t="n">
-        <v>813.33</v>
+        <v>135.7</v>
       </c>
       <c r="O5" t="n">
-        <v>821.67</v>
+        <v>136.5</v>
       </c>
       <c r="P5" t="n">
-        <v>830.83</v>
+        <v>137.4</v>
       </c>
       <c r="Q5" t="n">
-        <v>840</v>
+        <v>138.3</v>
       </c>
       <c r="R5" t="n">
-        <v>849.17</v>
-      </c>
-      <c r="S5" t="n">
-        <v>858.33</v>
-      </c>
-      <c r="T5" t="n">
-        <v>866.67</v>
-      </c>
-      <c r="U5" t="n">
-        <v>875.83</v>
-      </c>
-      <c r="V5" t="n">
-        <v>885</v>
-      </c>
-      <c r="W5" t="n">
-        <v>894.17</v>
-      </c>
-      <c r="X5" t="n">
-        <v>903.33</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Customer Care</t>
+          <t>Back Office</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -887,84 +820,66 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>240</v>
+        <v>105</v>
       </c>
       <c r="H6" t="n">
-        <v>243</v>
+        <v>106</v>
       </c>
       <c r="I6" t="n">
-        <v>246</v>
+        <v>107</v>
       </c>
       <c r="J6" t="n">
-        <v>249</v>
+        <v>108</v>
       </c>
       <c r="K6" t="n">
-        <v>252</v>
+        <v>109</v>
       </c>
       <c r="L6" t="n">
-        <v>254</v>
+        <v>109</v>
       </c>
       <c r="M6" t="n">
-        <v>257</v>
+        <v>110</v>
       </c>
       <c r="N6" t="n">
-        <v>260</v>
+        <v>111</v>
       </c>
       <c r="O6" t="n">
-        <v>263</v>
+        <v>112</v>
       </c>
       <c r="P6" t="n">
-        <v>266</v>
+        <v>113</v>
       </c>
       <c r="Q6" t="n">
-        <v>269</v>
+        <v>114</v>
       </c>
       <c r="R6" t="n">
-        <v>272</v>
-      </c>
-      <c r="S6" t="n">
-        <v>275</v>
-      </c>
-      <c r="T6" t="n">
-        <v>277</v>
-      </c>
-      <c r="U6" t="n">
-        <v>280</v>
-      </c>
-      <c r="V6" t="n">
-        <v>283</v>
-      </c>
-      <c r="W6" t="n">
-        <v>286</v>
-      </c>
-      <c r="X6" t="n">
-        <v>289</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Customer Care</t>
+          <t>Back Office</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -973,84 +888,66 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="H7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="I7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="J7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="M7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="N7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="O7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="P7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="R7" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="S7" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="T7" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="U7" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="V7" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="W7" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="X7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Customer Care</t>
+          <t>Back Office</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bali</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1059,84 +956,66 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>200</v>
+        <v>95.5</v>
       </c>
       <c r="H8" t="n">
-        <v>202.5</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>205</v>
+        <v>97.3</v>
       </c>
       <c r="J8" t="n">
-        <v>207.5</v>
+        <v>98.2</v>
       </c>
       <c r="K8" t="n">
-        <v>210</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>211.67</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>214.17</v>
+        <v>100</v>
       </c>
       <c r="N8" t="n">
-        <v>216.67</v>
+        <v>100.9</v>
       </c>
       <c r="O8" t="n">
-        <v>219.17</v>
+        <v>101.8</v>
       </c>
       <c r="P8" t="n">
-        <v>221.67</v>
+        <v>102.7</v>
       </c>
       <c r="Q8" t="n">
-        <v>224.17</v>
+        <v>103.6</v>
       </c>
       <c r="R8" t="n">
-        <v>226.67</v>
-      </c>
-      <c r="S8" t="n">
-        <v>229.17</v>
-      </c>
-      <c r="T8" t="n">
-        <v>230.83</v>
-      </c>
-      <c r="U8" t="n">
-        <v>233.33</v>
-      </c>
-      <c r="V8" t="n">
-        <v>235.83</v>
-      </c>
-      <c r="W8" t="n">
-        <v>238.33</v>
-      </c>
-      <c r="X8" t="n">
-        <v>240.83</v>
+        <v>104.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Escalations</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1145,84 +1024,66 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="H9" t="n">
-        <v>152</v>
+        <v>76</v>
       </c>
       <c r="I9" t="n">
-        <v>154</v>
+        <v>76</v>
       </c>
       <c r="J9" t="n">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="K9" t="n">
-        <v>157</v>
+        <v>78</v>
       </c>
       <c r="L9" t="n">
-        <v>159</v>
+        <v>79</v>
       </c>
       <c r="M9" t="n">
-        <v>161</v>
+        <v>79</v>
       </c>
       <c r="N9" t="n">
-        <v>163</v>
+        <v>80</v>
       </c>
       <c r="O9" t="n">
-        <v>164</v>
+        <v>81</v>
       </c>
       <c r="P9" t="n">
-        <v>166</v>
+        <v>81</v>
       </c>
       <c r="Q9" t="n">
-        <v>168</v>
+        <v>82</v>
       </c>
       <c r="R9" t="n">
-        <v>170</v>
-      </c>
-      <c r="S9" t="n">
-        <v>172</v>
-      </c>
-      <c r="T9" t="n">
-        <v>173</v>
-      </c>
-      <c r="U9" t="n">
-        <v>175</v>
-      </c>
-      <c r="V9" t="n">
-        <v>177</v>
-      </c>
-      <c r="W9" t="n">
-        <v>179</v>
-      </c>
-      <c r="X9" t="n">
-        <v>181</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Escalations</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1231,84 +1092,66 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="H10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="I10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="J10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="K10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="L10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="M10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="N10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="O10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
       <c r="R10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="S10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="T10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="U10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="V10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="W10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="X10" t="n">
-        <v>1.3</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Escalations</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Gurugram</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Surabaya</t>
+          <t>Aurora Park</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1317,84 +1160,66 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>115.38</v>
+        <v>60</v>
       </c>
       <c r="H11" t="n">
-        <v>116.92</v>
+        <v>60.8</v>
       </c>
       <c r="I11" t="n">
-        <v>118.46</v>
+        <v>60.8</v>
       </c>
       <c r="J11" t="n">
-        <v>119.23</v>
+        <v>61.6</v>
       </c>
       <c r="K11" t="n">
-        <v>120.77</v>
+        <v>62.4</v>
       </c>
       <c r="L11" t="n">
-        <v>122.31</v>
+        <v>63.2</v>
       </c>
       <c r="M11" t="n">
-        <v>123.85</v>
+        <v>63.2</v>
       </c>
       <c r="N11" t="n">
-        <v>125.38</v>
+        <v>64</v>
       </c>
       <c r="O11" t="n">
-        <v>126.15</v>
+        <v>64.8</v>
       </c>
       <c r="P11" t="n">
-        <v>127.69</v>
+        <v>64.8</v>
       </c>
       <c r="Q11" t="n">
-        <v>129.23</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="R11" t="n">
-        <v>130.77</v>
-      </c>
-      <c r="S11" t="n">
-        <v>132.31</v>
-      </c>
-      <c r="T11" t="n">
-        <v>133.08</v>
-      </c>
-      <c r="U11" t="n">
-        <v>134.62</v>
-      </c>
-      <c r="V11" t="n">
-        <v>136.15</v>
-      </c>
-      <c r="W11" t="n">
-        <v>137.69</v>
-      </c>
-      <c r="X11" t="n">
-        <v>139.23</v>
+        <v>66.40000000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Customer Care</t>
+          <t>Back Office</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Meridian One</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1403,84 +1228,66 @@
         </is>
       </c>
       <c r="G12" t="n">
+        <v>620</v>
+      </c>
+      <c r="H12" t="n">
+        <v>630</v>
+      </c>
+      <c r="I12" t="n">
         <v>640</v>
       </c>
-      <c r="H12" t="n">
-        <v>648</v>
-      </c>
-      <c r="I12" t="n">
-        <v>655</v>
-      </c>
       <c r="J12" t="n">
-        <v>663</v>
+        <v>650</v>
       </c>
       <c r="K12" t="n">
-        <v>671</v>
+        <v>660</v>
       </c>
       <c r="L12" t="n">
-        <v>678</v>
+        <v>670</v>
       </c>
       <c r="M12" t="n">
-        <v>686</v>
+        <v>680</v>
       </c>
       <c r="N12" t="n">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="O12" t="n">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="P12" t="n">
         <v>709</v>
       </c>
       <c r="Q12" t="n">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="R12" t="n">
-        <v>724</v>
-      </c>
-      <c r="S12" t="n">
-        <v>732</v>
-      </c>
-      <c r="T12" t="n">
-        <v>740</v>
-      </c>
-      <c r="U12" t="n">
-        <v>748</v>
-      </c>
-      <c r="V12" t="n">
-        <v>755</v>
-      </c>
-      <c r="W12" t="n">
-        <v>763</v>
-      </c>
-      <c r="X12" t="n">
-        <v>771</v>
+        <v>729</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Customer Care</t>
+          <t>Back Office</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Meridian One</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1524,49 +1331,31 @@
       <c r="R13" t="n">
         <v>1.1</v>
       </c>
-      <c r="S13" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="T13" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="U13" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="V13" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="W13" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="X13" t="n">
-        <v>1.1</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Customer Care</t>
+          <t>Back Office</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Meridian One</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1575,64 +1364,46 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>581.8200000000001</v>
+        <v>563.6</v>
       </c>
       <c r="H14" t="n">
-        <v>589.09</v>
+        <v>572.7</v>
       </c>
       <c r="I14" t="n">
-        <v>595.45</v>
+        <v>581.8</v>
       </c>
       <c r="J14" t="n">
-        <v>602.73</v>
+        <v>590.9</v>
       </c>
       <c r="K14" t="n">
-        <v>610</v>
+        <v>600</v>
       </c>
       <c r="L14" t="n">
-        <v>616.36</v>
+        <v>609.1</v>
       </c>
       <c r="M14" t="n">
-        <v>623.64</v>
+        <v>618.2</v>
       </c>
       <c r="N14" t="n">
-        <v>630.91</v>
+        <v>626.4</v>
       </c>
       <c r="O14" t="n">
-        <v>637.27</v>
+        <v>635.5</v>
       </c>
       <c r="P14" t="n">
-        <v>644.55</v>
+        <v>644.5</v>
       </c>
       <c r="Q14" t="n">
-        <v>651.8200000000001</v>
+        <v>653.6</v>
       </c>
       <c r="R14" t="n">
-        <v>658.1799999999999</v>
-      </c>
-      <c r="S14" t="n">
-        <v>665.45</v>
-      </c>
-      <c r="T14" t="n">
-        <v>672.73</v>
-      </c>
-      <c r="U14" t="n">
-        <v>680</v>
-      </c>
-      <c r="V14" t="n">
-        <v>686.36</v>
-      </c>
-      <c r="W14" t="n">
-        <v>693.64</v>
-      </c>
-      <c r="X14" t="n">
-        <v>700.91</v>
+        <v>662.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>Helio</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1642,17 +1413,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Skyline Center</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1661,64 +1432,46 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>160</v>
+        <v>560</v>
       </c>
       <c r="H15" t="n">
-        <v>162</v>
+        <v>575</v>
       </c>
       <c r="I15" t="n">
-        <v>164</v>
+        <v>589</v>
       </c>
       <c r="J15" t="n">
-        <v>166</v>
+        <v>604</v>
       </c>
       <c r="K15" t="n">
-        <v>168</v>
+        <v>618</v>
       </c>
       <c r="L15" t="n">
-        <v>170</v>
+        <v>633</v>
       </c>
       <c r="M15" t="n">
-        <v>172</v>
+        <v>647</v>
       </c>
       <c r="N15" t="n">
-        <v>173</v>
+        <v>662</v>
       </c>
       <c r="O15" t="n">
-        <v>175</v>
+        <v>676</v>
       </c>
       <c r="P15" t="n">
-        <v>177</v>
+        <v>691</v>
       </c>
       <c r="Q15" t="n">
-        <v>179</v>
+        <v>706</v>
       </c>
       <c r="R15" t="n">
-        <v>181</v>
-      </c>
-      <c r="S15" t="n">
-        <v>183</v>
-      </c>
-      <c r="T15" t="n">
-        <v>185</v>
-      </c>
-      <c r="U15" t="n">
-        <v>187</v>
-      </c>
-      <c r="V15" t="n">
-        <v>189</v>
-      </c>
-      <c r="W15" t="n">
-        <v>191</v>
-      </c>
-      <c r="X15" t="n">
-        <v>193</v>
+        <v>720</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>Helio</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1728,17 +1481,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Skyline Center</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1747,64 +1500,46 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="H16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="I16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="J16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="K16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="L16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="M16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="N16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="O16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="P16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="R16" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="S16" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="T16" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="U16" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="V16" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="W16" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="X16" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MI</t>
+          <t>Helio</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1814,17 +1549,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Skyline Center</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1833,64 +1568,46 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>145.45</v>
+        <v>466.7</v>
       </c>
       <c r="H17" t="n">
-        <v>147.27</v>
+        <v>479.2</v>
       </c>
       <c r="I17" t="n">
-        <v>149.09</v>
+        <v>490.8</v>
       </c>
       <c r="J17" t="n">
-        <v>150.91</v>
+        <v>503.3</v>
       </c>
       <c r="K17" t="n">
-        <v>152.73</v>
+        <v>515</v>
       </c>
       <c r="L17" t="n">
-        <v>154.55</v>
+        <v>527.5</v>
       </c>
       <c r="M17" t="n">
-        <v>156.36</v>
+        <v>539.2</v>
       </c>
       <c r="N17" t="n">
-        <v>157.27</v>
+        <v>551.7</v>
       </c>
       <c r="O17" t="n">
-        <v>159.09</v>
+        <v>563.3</v>
       </c>
       <c r="P17" t="n">
-        <v>160.91</v>
+        <v>575.8</v>
       </c>
       <c r="Q17" t="n">
-        <v>162.73</v>
+        <v>588.3</v>
       </c>
       <c r="R17" t="n">
-        <v>164.55</v>
-      </c>
-      <c r="S17" t="n">
-        <v>166.36</v>
-      </c>
-      <c r="T17" t="n">
-        <v>168.18</v>
-      </c>
-      <c r="U17" t="n">
-        <v>170</v>
-      </c>
-      <c r="V17" t="n">
-        <v>171.82</v>
-      </c>
-      <c r="W17" t="n">
-        <v>173.64</v>
-      </c>
-      <c r="X17" t="n">
-        <v>175.45</v>
+        <v>600</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>V2</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1900,17 +1617,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Skyline Center</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1919,64 +1636,46 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>230</v>
+        <v>640</v>
       </c>
       <c r="H18" t="n">
-        <v>233</v>
+        <v>659</v>
       </c>
       <c r="I18" t="n">
-        <v>236</v>
+        <v>678</v>
       </c>
       <c r="J18" t="n">
-        <v>238</v>
+        <v>698</v>
       </c>
       <c r="K18" t="n">
-        <v>241</v>
+        <v>717</v>
       </c>
       <c r="L18" t="n">
-        <v>244</v>
+        <v>736</v>
       </c>
       <c r="M18" t="n">
-        <v>247</v>
+        <v>755</v>
       </c>
       <c r="N18" t="n">
-        <v>249</v>
+        <v>774</v>
       </c>
       <c r="O18" t="n">
-        <v>252</v>
+        <v>794</v>
       </c>
       <c r="P18" t="n">
-        <v>255</v>
+        <v>813</v>
       </c>
       <c r="Q18" t="n">
-        <v>258</v>
+        <v>832</v>
       </c>
       <c r="R18" t="n">
-        <v>260</v>
-      </c>
-      <c r="S18" t="n">
-        <v>263</v>
-      </c>
-      <c r="T18" t="n">
-        <v>266</v>
-      </c>
-      <c r="U18" t="n">
-        <v>269</v>
-      </c>
-      <c r="V18" t="n">
-        <v>271</v>
-      </c>
-      <c r="W18" t="n">
-        <v>274</v>
-      </c>
-      <c r="X18" t="n">
-        <v>277</v>
+        <v>851</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>V2</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1986,17 +1685,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Skyline Center</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2038,31 +1737,13 @@
         <v>1.2</v>
       </c>
       <c r="R19" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="S19" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="T19" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="U19" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="V19" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="W19" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="X19" t="n">
         <v>1.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>V2</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2072,17 +1753,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Skyline Center</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2091,64 +1772,46 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>191.67</v>
+        <v>533.3</v>
       </c>
       <c r="H20" t="n">
-        <v>194.17</v>
+        <v>549.2</v>
       </c>
       <c r="I20" t="n">
-        <v>196.67</v>
+        <v>565</v>
       </c>
       <c r="J20" t="n">
-        <v>198.33</v>
+        <v>581.7</v>
       </c>
       <c r="K20" t="n">
-        <v>200.83</v>
+        <v>597.5</v>
       </c>
       <c r="L20" t="n">
-        <v>203.33</v>
+        <v>613.3</v>
       </c>
       <c r="M20" t="n">
-        <v>205.83</v>
+        <v>629.2</v>
       </c>
       <c r="N20" t="n">
-        <v>207.5</v>
+        <v>645</v>
       </c>
       <c r="O20" t="n">
-        <v>210</v>
+        <v>661.7</v>
       </c>
       <c r="P20" t="n">
-        <v>212.5</v>
+        <v>677.5</v>
       </c>
       <c r="Q20" t="n">
-        <v>215</v>
+        <v>693.3</v>
       </c>
       <c r="R20" t="n">
-        <v>216.67</v>
-      </c>
-      <c r="S20" t="n">
-        <v>219.17</v>
-      </c>
-      <c r="T20" t="n">
-        <v>221.67</v>
-      </c>
-      <c r="U20" t="n">
-        <v>224.17</v>
-      </c>
-      <c r="V20" t="n">
-        <v>225.83</v>
-      </c>
-      <c r="W20" t="n">
-        <v>228.33</v>
-      </c>
-      <c r="X20" t="n">
-        <v>230.83</v>
+        <v>709.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2158,17 +1821,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Danang</t>
+          <t>Cebu</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Danang</t>
+          <t>Harbour Point</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2177,64 +1840,46 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>520</v>
+        <v>230</v>
       </c>
       <c r="H21" t="n">
-        <v>526</v>
+        <v>234</v>
       </c>
       <c r="I21" t="n">
-        <v>532</v>
+        <v>238</v>
       </c>
       <c r="J21" t="n">
-        <v>539</v>
+        <v>242</v>
       </c>
       <c r="K21" t="n">
-        <v>545</v>
+        <v>247</v>
       </c>
       <c r="L21" t="n">
-        <v>551</v>
+        <v>251</v>
       </c>
       <c r="M21" t="n">
-        <v>557</v>
+        <v>255</v>
       </c>
       <c r="N21" t="n">
-        <v>564</v>
+        <v>259</v>
       </c>
       <c r="O21" t="n">
-        <v>570</v>
+        <v>263</v>
       </c>
       <c r="P21" t="n">
-        <v>576</v>
+        <v>267</v>
       </c>
       <c r="Q21" t="n">
-        <v>582</v>
+        <v>271</v>
       </c>
       <c r="R21" t="n">
-        <v>589</v>
-      </c>
-      <c r="S21" t="n">
-        <v>595</v>
-      </c>
-      <c r="T21" t="n">
-        <v>601</v>
-      </c>
-      <c r="U21" t="n">
-        <v>607</v>
-      </c>
-      <c r="V21" t="n">
-        <v>614</v>
-      </c>
-      <c r="W21" t="n">
-        <v>620</v>
-      </c>
-      <c r="X21" t="n">
-        <v>626</v>
+        <v>276</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2244,17 +1889,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Danang</t>
+          <t>Cebu</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Danang</t>
+          <t>Harbour Point</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2296,31 +1941,13 @@
         <v>1.2</v>
       </c>
       <c r="R22" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="S22" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="T22" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="U22" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="V22" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="W22" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="X22" t="n">
         <v>1.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Nimbus</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2330,17 +1957,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Danang</t>
+          <t>Cebu</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Danang</t>
+          <t>Harbour Point</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2349,84 +1976,66 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>433.33</v>
+        <v>191.7</v>
       </c>
       <c r="H23" t="n">
-        <v>438.33</v>
+        <v>195</v>
       </c>
       <c r="I23" t="n">
-        <v>443.33</v>
+        <v>198.3</v>
       </c>
       <c r="J23" t="n">
-        <v>449.17</v>
+        <v>201.7</v>
       </c>
       <c r="K23" t="n">
-        <v>454.17</v>
+        <v>205.8</v>
       </c>
       <c r="L23" t="n">
-        <v>459.17</v>
+        <v>209.2</v>
       </c>
       <c r="M23" t="n">
-        <v>464.17</v>
+        <v>212.5</v>
       </c>
       <c r="N23" t="n">
-        <v>470</v>
+        <v>215.8</v>
       </c>
       <c r="O23" t="n">
-        <v>475</v>
+        <v>219.2</v>
       </c>
       <c r="P23" t="n">
-        <v>480</v>
+        <v>222.5</v>
       </c>
       <c r="Q23" t="n">
-        <v>485</v>
+        <v>225.8</v>
       </c>
       <c r="R23" t="n">
-        <v>490.83</v>
-      </c>
-      <c r="S23" t="n">
-        <v>495.83</v>
-      </c>
-      <c r="T23" t="n">
-        <v>500.83</v>
-      </c>
-      <c r="U23" t="n">
-        <v>505.83</v>
-      </c>
-      <c r="V23" t="n">
-        <v>511.67</v>
-      </c>
-      <c r="W23" t="n">
-        <v>516.67</v>
-      </c>
-      <c r="X23" t="n">
-        <v>521.67</v>
+        <v>230</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Back Office</t>
+          <t>Collections</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Krakow</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Vistula House</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2435,84 +2044,66 @@
         </is>
       </c>
       <c r="G24" t="n">
+        <v>300</v>
+      </c>
+      <c r="H24" t="n">
+        <v>306</v>
+      </c>
+      <c r="I24" t="n">
+        <v>312</v>
+      </c>
+      <c r="J24" t="n">
+        <v>318</v>
+      </c>
+      <c r="K24" t="n">
+        <v>324</v>
+      </c>
+      <c r="L24" t="n">
         <v>330</v>
       </c>
-      <c r="H24" t="n">
-        <v>334</v>
-      </c>
-      <c r="I24" t="n">
-        <v>338</v>
-      </c>
-      <c r="J24" t="n">
+      <c r="M24" t="n">
+        <v>336</v>
+      </c>
+      <c r="N24" t="n">
         <v>342</v>
       </c>
-      <c r="K24" t="n">
-        <v>346</v>
-      </c>
-      <c r="L24" t="n">
-        <v>350</v>
-      </c>
-      <c r="M24" t="n">
+      <c r="O24" t="n">
+        <v>348</v>
+      </c>
+      <c r="P24" t="n">
         <v>354</v>
       </c>
-      <c r="N24" t="n">
-        <v>358</v>
-      </c>
-      <c r="O24" t="n">
-        <v>362</v>
-      </c>
-      <c r="P24" t="n">
+      <c r="Q24" t="n">
+        <v>360</v>
+      </c>
+      <c r="R24" t="n">
         <v>366</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>370</v>
-      </c>
-      <c r="R24" t="n">
-        <v>374</v>
-      </c>
-      <c r="S24" t="n">
-        <v>378</v>
-      </c>
-      <c r="T24" t="n">
-        <v>381</v>
-      </c>
-      <c r="U24" t="n">
-        <v>385</v>
-      </c>
-      <c r="V24" t="n">
-        <v>389</v>
-      </c>
-      <c r="W24" t="n">
-        <v>393</v>
-      </c>
-      <c r="X24" t="n">
-        <v>397</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Back Office</t>
+          <t>Collections</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Krakow</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Vistula House</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2521,84 +2112,66 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="K25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="L25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="N25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="O25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="P25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="R25" t="n">
-        <v>1</v>
-      </c>
-      <c r="S25" t="n">
-        <v>1</v>
-      </c>
-      <c r="T25" t="n">
-        <v>1</v>
-      </c>
-      <c r="U25" t="n">
-        <v>1</v>
-      </c>
-      <c r="V25" t="n">
-        <v>1</v>
-      </c>
-      <c r="W25" t="n">
-        <v>1</v>
-      </c>
-      <c r="X25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TNS</t>
+          <t>Vector</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Back Office</t>
+          <t>Collections</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Krakow</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Vistula House</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2607,58 +2180,244 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>330</v>
+        <v>240</v>
       </c>
       <c r="H26" t="n">
-        <v>334</v>
+        <v>244.8</v>
       </c>
       <c r="I26" t="n">
-        <v>338</v>
+        <v>249.6</v>
       </c>
       <c r="J26" t="n">
-        <v>342</v>
+        <v>254.4</v>
       </c>
       <c r="K26" t="n">
-        <v>346</v>
+        <v>259.2</v>
       </c>
       <c r="L26" t="n">
-        <v>350</v>
+        <v>264</v>
       </c>
       <c r="M26" t="n">
-        <v>354</v>
+        <v>268.8</v>
       </c>
       <c r="N26" t="n">
-        <v>358</v>
+        <v>273.6</v>
       </c>
       <c r="O26" t="n">
-        <v>362</v>
+        <v>278.4</v>
       </c>
       <c r="P26" t="n">
-        <v>366</v>
+        <v>283.2</v>
       </c>
       <c r="Q26" t="n">
-        <v>370</v>
+        <v>288</v>
       </c>
       <c r="R26" t="n">
-        <v>374</v>
-      </c>
-      <c r="S26" t="n">
-        <v>378</v>
-      </c>
-      <c r="T26" t="n">
-        <v>381</v>
-      </c>
-      <c r="U26" t="n">
-        <v>385</v>
-      </c>
-      <c r="V26" t="n">
-        <v>389</v>
-      </c>
-      <c r="W26" t="n">
-        <v>393</v>
-      </c>
-      <c r="X26" t="n">
-        <v>397</v>
+        <v>292.8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nimbus</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Escalations</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Krakow</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Vistula House</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>HC Forecast</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>95</v>
+      </c>
+      <c r="H27" t="n">
+        <v>96</v>
+      </c>
+      <c r="I27" t="n">
+        <v>98</v>
+      </c>
+      <c r="J27" t="n">
+        <v>99</v>
+      </c>
+      <c r="K27" t="n">
+        <v>100</v>
+      </c>
+      <c r="L27" t="n">
+        <v>102</v>
+      </c>
+      <c r="M27" t="n">
+        <v>103</v>
+      </c>
+      <c r="N27" t="n">
+        <v>104</v>
+      </c>
+      <c r="O27" t="n">
+        <v>106</v>
+      </c>
+      <c r="P27" t="n">
+        <v>107</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>108</v>
+      </c>
+      <c r="R27" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Nimbus</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Escalations</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Krakow</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Vistula House</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Seat Ratio</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="O28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Nimbus</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Escalations</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Krakow</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Vistula House</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Seats Required</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>76</v>
+      </c>
+      <c r="H29" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="I29" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="J29" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="K29" t="n">
+        <v>80</v>
+      </c>
+      <c r="L29" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M29" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="N29" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="O29" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="P29" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="R29" t="n">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>